<commit_message>
updated to account for overhead
</commit_message>
<xml_diff>
--- a/hwo_star_list_for_neid.xlsx
+++ b/hwo_star_list_for_neid.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8BDD3B59D38335A8/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shire\eprv-survey-simulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DD456C0-18F6-4BA9-9193-A0CC545D6A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67D5348-8F3B-4880-96EE-C1558E2ED18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9975979B-17AC-4192-86B9-BD5B2BA3458A}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3910" uniqueCount="1383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4075" uniqueCount="1544">
   <si>
     <t>rowid</t>
   </si>
@@ -4169,6 +4169,489 @@
   </si>
   <si>
     <t>03091+4937</t>
+  </si>
+  <si>
+    <t>OscTime_10cms</t>
+  </si>
+  <si>
+    <t>390.65085449999907</t>
+  </si>
+  <si>
+    <t>966.2658569999969</t>
+  </si>
+  <si>
+    <t>8660.21712</t>
+  </si>
+  <si>
+    <t>4714.9653299999745</t>
+  </si>
+  <si>
+    <t>1533.5984850000002</t>
+  </si>
+  <si>
+    <t>16575.15480000001</t>
+  </si>
+  <si>
+    <t>136.75167600000012</t>
+  </si>
+  <si>
+    <t>4404.440190000003</t>
+  </si>
+  <si>
+    <t>943.2110369999988</t>
+  </si>
+  <si>
+    <t>11838.10463999997</t>
+  </si>
+  <si>
+    <t>4067.5036950000003</t>
+  </si>
+  <si>
+    <t>224.41881749999985</t>
+  </si>
+  <si>
+    <t>682.9470224999992</t>
+  </si>
+  <si>
+    <t>6753.741465000008</t>
+  </si>
+  <si>
+    <t>5176.110449999999</t>
+  </si>
+  <si>
+    <t>581.8488194999991</t>
+  </si>
+  <si>
+    <t>158.25650250000004</t>
+  </si>
+  <si>
+    <t>191.83630949999974</t>
+  </si>
+  <si>
+    <t>4435.776510000011</t>
+  </si>
+  <si>
+    <t>2346.8365049999984</t>
+  </si>
+  <si>
+    <t>694.5899999999991</t>
+  </si>
+  <si>
+    <t>192.867309</t>
+  </si>
+  <si>
+    <t>2197.4510399999976</t>
+  </si>
+  <si>
+    <t>4012.959930000001</t>
+  </si>
+  <si>
+    <t>866.3605544999966</t>
+  </si>
+  <si>
+    <t>2140.7847899999856</t>
+  </si>
+  <si>
+    <t>190.34344500000046</t>
+  </si>
+  <si>
+    <t>384.36777300000045</t>
+  </si>
+  <si>
+    <t>4174.0853099999795</t>
+  </si>
+  <si>
+    <t>3541.1660699999893</t>
+  </si>
+  <si>
+    <t>3592.9999949999883</t>
+  </si>
+  <si>
+    <t>241.41460949999947</t>
+  </si>
+  <si>
+    <t>1865.2327949999894</t>
+  </si>
+  <si>
+    <t>154.3458914999997</t>
+  </si>
+  <si>
+    <t>209.30164649999986</t>
+  </si>
+  <si>
+    <t>190.14506400000005</t>
+  </si>
+  <si>
+    <t>2512.502384999991</t>
+  </si>
+  <si>
+    <t>11092.814579999971</t>
+  </si>
+  <si>
+    <t>259.60234050000014</t>
+  </si>
+  <si>
+    <t>279.5131229999999</t>
+  </si>
+  <si>
+    <t>6396.657915000033</t>
+  </si>
+  <si>
+    <t>192.2668634999998</t>
+  </si>
+  <si>
+    <t>386.956278</t>
+  </si>
+  <si>
+    <t>1508.9302950000003</t>
+  </si>
+  <si>
+    <t>2555.551829999992</t>
+  </si>
+  <si>
+    <t>1937.185664999993</t>
+  </si>
+  <si>
+    <t>147.7631880000002</t>
+  </si>
+  <si>
+    <t>1518.5991300000012</t>
+  </si>
+  <si>
+    <t>1533.4841249999974</t>
+  </si>
+  <si>
+    <t>1016.2589729999966</t>
+  </si>
+  <si>
+    <t>8164.976550000018</t>
+  </si>
+  <si>
+    <t>1048.729742999997</t>
+  </si>
+  <si>
+    <t>1655.144474999997</t>
+  </si>
+  <si>
+    <t>2261.1316949999973</t>
+  </si>
+  <si>
+    <t>3897.6470249999993</t>
+  </si>
+  <si>
+    <t>112.14922950000064</t>
+  </si>
+  <si>
+    <t>144.58012500000004</t>
+  </si>
+  <si>
+    <t>3415.8156449999933</t>
+  </si>
+  <si>
+    <t>306.6500460000007</t>
+  </si>
+  <si>
+    <t>288.28397250000074</t>
+  </si>
+  <si>
+    <t>1011.4437449999992</t>
+  </si>
+  <si>
+    <t>4292.142224999995</t>
+  </si>
+  <si>
+    <t>344.3493000000014</t>
+  </si>
+  <si>
+    <t>2908.2915149999985</t>
+  </si>
+  <si>
+    <t>112.74241350000057</t>
+  </si>
+  <si>
+    <t>207.46151999999998</t>
+  </si>
+  <si>
+    <t>229.10685600000033</t>
+  </si>
+  <si>
+    <t>148.07862450000005</t>
+  </si>
+  <si>
+    <t>661.7869439999992</t>
+  </si>
+  <si>
+    <t>2947.946759999995</t>
+  </si>
+  <si>
+    <t>3530.9857199999933</t>
+  </si>
+  <si>
+    <t>227.95443450000016</t>
+  </si>
+  <si>
+    <t>4944.132825000003</t>
+  </si>
+  <si>
+    <t>130.87842600000056</t>
+  </si>
+  <si>
+    <t>179.13006299999952</t>
+  </si>
+  <si>
+    <t>210.05474999999944</t>
+  </si>
+  <si>
+    <t>4280.343000000011</t>
+  </si>
+  <si>
+    <t>4282.392104999999</t>
+  </si>
+  <si>
+    <t>4544.636625000011</t>
+  </si>
+  <si>
+    <t>362.2343445000009</t>
+  </si>
+  <si>
+    <t>6777.680925000024</t>
+  </si>
+  <si>
+    <t>203.59915949999973</t>
+  </si>
+  <si>
+    <t>394.09693950000013</t>
+  </si>
+  <si>
+    <t>200.83430550000065</t>
+  </si>
+  <si>
+    <t>4164.037500000008</t>
+  </si>
+  <si>
+    <t>4902.5679600000185</t>
+  </si>
+  <si>
+    <t>8078.283120000015</t>
+  </si>
+  <si>
+    <t>3172.5781199999974</t>
+  </si>
+  <si>
+    <t>3389.387954999994</t>
+  </si>
+  <si>
+    <t>2146.994159999987</t>
+  </si>
+  <si>
+    <t>161.50753200000045</t>
+  </si>
+  <si>
+    <t>203.83682399999964</t>
+  </si>
+  <si>
+    <t>1056.5292734999991</t>
+  </si>
+  <si>
+    <t>205.1840310000007</t>
+  </si>
+  <si>
+    <t>1927.8064799999906</t>
+  </si>
+  <si>
+    <t>2019.6637949999956</t>
+  </si>
+  <si>
+    <t>263.2702454999998</t>
+  </si>
+  <si>
+    <t>3108.2241299999964</t>
+  </si>
+  <si>
+    <t>2899.7662649999975</t>
+  </si>
+  <si>
+    <t>1616.4264299999977</t>
+  </si>
+  <si>
+    <t>230.81567399999958</t>
+  </si>
+  <si>
+    <t>1859.0919449999913</t>
+  </si>
+  <si>
+    <t>1026.9954674999976</t>
+  </si>
+  <si>
+    <t>2322.3437849999877</t>
+  </si>
+  <si>
+    <t>2516.8605449999914</t>
+  </si>
+  <si>
+    <t>1474.1961254999997</t>
+  </si>
+  <si>
+    <t>5265.90063</t>
+  </si>
+  <si>
+    <t>140.69691900000015</t>
+  </si>
+  <si>
+    <t>3587.5097399999977</t>
+  </si>
+  <si>
+    <t>1370.8638749999973</t>
+  </si>
+  <si>
+    <t>293.3419665000012</t>
+  </si>
+  <si>
+    <t>1148.7534989999979</t>
+  </si>
+  <si>
+    <t>148.7238404999999</t>
+  </si>
+  <si>
+    <t>5811.202274999998</t>
+  </si>
+  <si>
+    <t>3642.8356949999916</t>
+  </si>
+  <si>
+    <t>5344.188689999996</t>
+  </si>
+  <si>
+    <t>2058.221129999989</t>
+  </si>
+  <si>
+    <t>2182.775999999989</t>
+  </si>
+  <si>
+    <t>1298.5357049999961</t>
+  </si>
+  <si>
+    <t>152.20717650000017</t>
+  </si>
+  <si>
+    <t>182.28788849999998</t>
+  </si>
+  <si>
+    <t>209.25814199999928</t>
+  </si>
+  <si>
+    <t>297.61656000000124</t>
+  </si>
+  <si>
+    <t>161.82402</t>
+  </si>
+  <si>
+    <t>202.29625349999966</t>
+  </si>
+  <si>
+    <t>2981.440079999994</t>
+  </si>
+  <si>
+    <t>149.81932950000078</t>
+  </si>
+  <si>
+    <t>149.28071549999993</t>
+  </si>
+  <si>
+    <t>202.42650599999934</t>
+  </si>
+  <si>
+    <t>640.6630305000008</t>
+  </si>
+  <si>
+    <t>289.7713424999996</t>
+  </si>
+  <si>
+    <t>11545.696799999982</t>
+  </si>
+  <si>
+    <t>296.72803949999957</t>
+  </si>
+  <si>
+    <t>307.4587980000007</t>
+  </si>
+  <si>
+    <t>1744.2433349999935</t>
+  </si>
+  <si>
+    <t>1229.9944200000016</t>
+  </si>
+  <si>
+    <t>188.47602299999966</t>
+  </si>
+  <si>
+    <t>3444.4542299999816</t>
+  </si>
+  <si>
+    <t>1957.635869999992</t>
+  </si>
+  <si>
+    <t>932.5661955000006</t>
+  </si>
+  <si>
+    <t>1100.7933119999952</t>
+  </si>
+  <si>
+    <t>7737.787665000022</t>
+  </si>
+  <si>
+    <t>228.06934350000006</t>
+  </si>
+  <si>
+    <t>856.3013834999986</t>
+  </si>
+  <si>
+    <t>5449.444995000004</t>
+  </si>
+  <si>
+    <t>900.2094479999964</t>
+  </si>
+  <si>
+    <t>183.56969699999962</t>
+  </si>
+  <si>
+    <t>329.7436875000004</t>
+  </si>
+  <si>
+    <t>3890.070570000003</t>
+  </si>
+  <si>
+    <t>112.95082950000052</t>
+  </si>
+  <si>
+    <t>1579.4301149999947</t>
+  </si>
+  <si>
+    <t>4974.957480000006</t>
+  </si>
+  <si>
+    <t>182.15289899999973</t>
+  </si>
+  <si>
+    <t>5582.053709999994</t>
+  </si>
+  <si>
+    <t>5877.7173300000195</t>
+  </si>
+  <si>
+    <t>1408.0462604999987</t>
+  </si>
+  <si>
+    <t>1035.1046294999987</t>
+  </si>
+  <si>
+    <t>6398.299529999997</t>
+  </si>
+  <si>
+    <t>8957.851545000016</t>
+  </si>
+  <si>
+    <t>3153.9800999999948</t>
   </si>
 </sst>
 </file>
@@ -5030,10 +5513,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0751AF21-EB19-499A-8E64-939139CBEE28}">
-  <dimension ref="A1:BH165"/>
+  <dimension ref="A1:BI165"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5214,8 +5697,11 @@
       <c r="BH1" t="s">
         <v>59</v>
       </c>
+      <c r="BI1" t="s">
+        <v>1383</v>
+      </c>
     </row>
-    <row r="2" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5381,8 +5867,11 @@
       <c r="BH2">
         <v>9.6</v>
       </c>
+      <c r="BI2" t="s">
+        <v>1384</v>
+      </c>
     </row>
-    <row r="3" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5542,8 +6031,11 @@
       <c r="BH3">
         <v>2.5</v>
       </c>
+      <c r="BI3" t="s">
+        <v>1385</v>
+      </c>
     </row>
-    <row r="4" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5721,8 +6213,11 @@
       <c r="BH4">
         <v>5.8</v>
       </c>
+      <c r="BI4" t="s">
+        <v>1386</v>
+      </c>
     </row>
-    <row r="5" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5882,8 +6377,11 @@
       <c r="BH5">
         <v>2.2000000000000002</v>
       </c>
+      <c r="BI5" t="s">
+        <v>1387</v>
+      </c>
     </row>
-    <row r="6" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -6061,8 +6559,11 @@
       <c r="BH6">
         <v>2.1</v>
       </c>
+      <c r="BI6" t="s">
+        <v>1388</v>
+      </c>
     </row>
-    <row r="7" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6234,8 +6735,11 @@
       <c r="BH7">
         <v>2</v>
       </c>
+      <c r="BI7" t="s">
+        <v>1389</v>
+      </c>
     </row>
-    <row r="8" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -6398,8 +6902,11 @@
       <c r="BH8">
         <v>0.5</v>
       </c>
+      <c r="BI8" t="s">
+        <v>1390</v>
+      </c>
     </row>
-    <row r="9" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -6577,8 +7084,11 @@
       <c r="BH9">
         <v>66.8</v>
       </c>
+      <c r="BI9" t="s">
+        <v>1391</v>
+      </c>
     </row>
-    <row r="10" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -6753,8 +7263,11 @@
       <c r="BH10">
         <v>0.1</v>
       </c>
+      <c r="BI10" t="s">
+        <v>1392</v>
+      </c>
     </row>
-    <row r="11" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -6914,8 +7427,11 @@
       <c r="BH11">
         <v>4.3360000000000003</v>
       </c>
+      <c r="BI11" t="s">
+        <v>1393</v>
+      </c>
     </row>
-    <row r="12" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -7093,8 +7609,11 @@
       <c r="BH12">
         <v>2</v>
       </c>
+      <c r="BI12" t="s">
+        <v>1394</v>
+      </c>
     </row>
-    <row r="13" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -7272,8 +7791,11 @@
       <c r="BH13">
         <v>4.4000000000000004</v>
       </c>
+      <c r="BI13" t="s">
+        <v>1395</v>
+      </c>
     </row>
-    <row r="14" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -7436,8 +7958,11 @@
       <c r="BH14">
         <v>2.3679999999999999</v>
       </c>
+      <c r="BI14" t="s">
+        <v>1396</v>
+      </c>
     </row>
-    <row r="15" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -7600,8 +8125,11 @@
       <c r="BH15">
         <v>2.8</v>
       </c>
+      <c r="BI15" t="s">
+        <v>1397</v>
+      </c>
     </row>
-    <row r="16" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -7776,8 +8304,11 @@
       <c r="BH16">
         <v>2</v>
       </c>
+      <c r="BI16" t="s">
+        <v>1398</v>
+      </c>
     </row>
-    <row r="17" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -7949,8 +8480,11 @@
       <c r="BH17">
         <v>3.6890000000000001</v>
       </c>
+      <c r="BI17" t="s">
+        <v>1399</v>
+      </c>
     </row>
-    <row r="18" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -8125,8 +8659,11 @@
       <c r="BH18">
         <v>0.9</v>
       </c>
+      <c r="BI18" t="s">
+        <v>1400</v>
+      </c>
     </row>
-    <row r="19" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -8304,8 +8841,11 @@
       <c r="BH19">
         <v>1.97</v>
       </c>
+      <c r="BI19" t="s">
+        <v>1401</v>
+      </c>
     </row>
-    <row r="20" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -8477,8 +9017,11 @@
       <c r="BH20">
         <v>18.899999999999999</v>
       </c>
+      <c r="BI20" t="s">
+        <v>1402</v>
+      </c>
     </row>
-    <row r="21" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -8641,8 +9184,11 @@
       <c r="BH21">
         <v>4.2569999999999997</v>
       </c>
+      <c r="BI21" t="s">
+        <v>1403</v>
+      </c>
     </row>
-    <row r="22" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -8817,8 +9363,11 @@
       <c r="BH22">
         <v>7.3</v>
       </c>
+      <c r="BI22" t="s">
+        <v>1404</v>
+      </c>
     </row>
-    <row r="23" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -8990,8 +9539,11 @@
       <c r="BH23">
         <v>0.1</v>
       </c>
+      <c r="BI23" t="s">
+        <v>1405</v>
+      </c>
     </row>
-    <row r="24" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -9166,8 +9718,11 @@
       <c r="BH24">
         <v>1.3</v>
       </c>
+      <c r="BI24" t="s">
+        <v>1406</v>
+      </c>
     </row>
-    <row r="25" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -9345,8 +9900,11 @@
       <c r="BH25">
         <v>8.8000000000000007</v>
       </c>
+      <c r="BI25" t="s">
+        <v>1407</v>
+      </c>
     </row>
-    <row r="26" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -9506,8 +10064,11 @@
       <c r="BH26">
         <v>1.3</v>
       </c>
+      <c r="BI26" t="s">
+        <v>1408</v>
+      </c>
     </row>
-    <row r="27" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -9670,8 +10231,11 @@
       <c r="BH27">
         <v>2</v>
       </c>
+      <c r="BI27" t="s">
+        <v>1409</v>
+      </c>
     </row>
-    <row r="28" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -9846,8 +10410,11 @@
       <c r="BH28">
         <v>1.6</v>
       </c>
+      <c r="BI28" t="s">
+        <v>1410</v>
+      </c>
     </row>
-    <row r="29" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -10022,8 +10589,11 @@
       <c r="BH29">
         <v>2.2130000000000001</v>
       </c>
+      <c r="BI29" t="s">
+        <v>1411</v>
+      </c>
     </row>
-    <row r="30" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -10198,8 +10768,11 @@
       <c r="BH30">
         <v>2.8</v>
       </c>
+      <c r="BI30" t="s">
+        <v>1412</v>
+      </c>
     </row>
-    <row r="31" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -10377,8 +10950,11 @@
       <c r="BH31">
         <v>34.700000000000003</v>
       </c>
+      <c r="BI31" t="s">
+        <v>1413</v>
+      </c>
     </row>
-    <row r="32" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -10541,8 +11117,11 @@
       <c r="BH32">
         <v>10</v>
       </c>
+      <c r="BI32" t="s">
+        <v>1414</v>
+      </c>
     </row>
-    <row r="33" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -10720,8 +11299,11 @@
       <c r="BH33">
         <v>1.8</v>
       </c>
+      <c r="BI33" t="s">
+        <v>1415</v>
+      </c>
     </row>
-    <row r="34" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -10884,8 +11466,11 @@
       <c r="BH34">
         <v>3.9</v>
       </c>
+      <c r="BI34" t="s">
+        <v>1416</v>
+      </c>
     </row>
-    <row r="35" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -11063,8 +11648,11 @@
       <c r="BH35">
         <v>2.54</v>
       </c>
+      <c r="BI35" t="s">
+        <v>1417</v>
+      </c>
     </row>
-    <row r="36" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -11239,8 +11827,11 @@
       <c r="BH36">
         <v>0.1</v>
       </c>
+      <c r="BI36" t="s">
+        <v>1418</v>
+      </c>
     </row>
-    <row r="37" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -11400,8 +11991,11 @@
       <c r="BH37">
         <v>1.821</v>
       </c>
+      <c r="BI37" t="s">
+        <v>1419</v>
+      </c>
     </row>
-    <row r="38" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -11579,8 +12173,11 @@
       <c r="BH38">
         <v>8</v>
       </c>
+      <c r="BI38" t="s">
+        <v>1420</v>
+      </c>
     </row>
-    <row r="39" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -11758,8 +12355,11 @@
       <c r="BH39">
         <v>5.0609999999999999</v>
       </c>
+      <c r="BI39" t="s">
+        <v>1421</v>
+      </c>
     </row>
-    <row r="40" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -11934,8 +12534,11 @@
       <c r="BH40">
         <v>2.7610000000000001</v>
       </c>
+      <c r="BI40" t="s">
+        <v>1422</v>
+      </c>
     </row>
-    <row r="41" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -12101,8 +12704,11 @@
       <c r="BH41">
         <v>2.069</v>
       </c>
+      <c r="BI41" t="s">
+        <v>1423</v>
+      </c>
     </row>
-    <row r="42" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -12265,8 +12871,11 @@
       <c r="BH42">
         <v>14</v>
       </c>
+      <c r="BI42" t="s">
+        <v>1424</v>
+      </c>
     </row>
-    <row r="43" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -12444,8 +13053,11 @@
       <c r="BH43">
         <v>2.11</v>
       </c>
+      <c r="BI43" t="s">
+        <v>1425</v>
+      </c>
     </row>
-    <row r="44" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -12611,8 +13223,11 @@
       <c r="BH44">
         <v>4.3710000000000004</v>
       </c>
+      <c r="BI44" t="s">
+        <v>1426</v>
+      </c>
     </row>
-    <row r="45" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -12778,8 +13393,11 @@
       <c r="BH45">
         <v>4.633</v>
       </c>
+      <c r="BI45" t="s">
+        <v>1427</v>
+      </c>
     </row>
-    <row r="46" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -12957,8 +13575,11 @@
       <c r="BH46">
         <v>7.2</v>
       </c>
+      <c r="BI46" t="s">
+        <v>1428</v>
+      </c>
     </row>
-    <row r="47" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -13136,8 +13757,11 @@
       <c r="BH47">
         <v>3.8</v>
       </c>
+      <c r="BI47" t="s">
+        <v>1429</v>
+      </c>
     </row>
-    <row r="48" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -13309,8 +13933,11 @@
       <c r="BH48">
         <v>2.9049999999999998</v>
       </c>
+      <c r="BI48" t="s">
+        <v>1430</v>
+      </c>
     </row>
-    <row r="49" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -13482,8 +14109,11 @@
       <c r="BH49">
         <v>2.569</v>
       </c>
+      <c r="BI49" t="s">
+        <v>1431</v>
+      </c>
     </row>
-    <row r="50" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -13643,8 +14273,11 @@
       <c r="BH50">
         <v>0.1</v>
       </c>
+      <c r="BI50" t="s">
+        <v>1432</v>
+      </c>
     </row>
-    <row r="51" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -13819,8 +14452,11 @@
       <c r="BH51">
         <v>2.855</v>
       </c>
+      <c r="BI51" t="s">
+        <v>1433</v>
+      </c>
     </row>
-    <row r="52" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -13995,8 +14631,11 @@
       <c r="BH52">
         <v>61.1</v>
       </c>
+      <c r="BI52" t="s">
+        <v>1434</v>
+      </c>
     </row>
-    <row r="53" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -14159,8 +14798,11 @@
       <c r="BH53">
         <v>3.6360000000000001</v>
       </c>
+      <c r="BI53" t="s">
+        <v>1435</v>
+      </c>
     </row>
-    <row r="54" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -14335,8 +14977,11 @@
       <c r="BH54">
         <v>0.9</v>
       </c>
+      <c r="BI54" t="s">
+        <v>1436</v>
+      </c>
     </row>
-    <row r="55" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -14511,8 +15156,11 @@
       <c r="BH55">
         <v>0.1</v>
       </c>
+      <c r="BI55" t="s">
+        <v>1437</v>
+      </c>
     </row>
-    <row r="56" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -14690,8 +15338,11 @@
       <c r="BH56">
         <v>5.55</v>
       </c>
+      <c r="BI56" t="s">
+        <v>1438</v>
+      </c>
     </row>
-    <row r="57" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -14845,8 +15496,11 @@
       <c r="BH57">
         <v>0.9</v>
       </c>
+      <c r="BI57" t="s">
+        <v>1439</v>
+      </c>
     </row>
-    <row r="58" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -15012,8 +15666,11 @@
       <c r="BH58">
         <v>1.9510000000000001</v>
       </c>
+      <c r="BI58" t="s">
+        <v>1440</v>
+      </c>
     </row>
-    <row r="59" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -15188,8 +15845,11 @@
       <c r="BH59">
         <v>16.399999999999999</v>
       </c>
+      <c r="BI59" t="s">
+        <v>1441</v>
+      </c>
     </row>
-    <row r="60" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -15367,8 +16027,11 @@
       <c r="BH60">
         <v>1.7</v>
       </c>
+      <c r="BI60" t="s">
+        <v>1442</v>
+      </c>
     </row>
-    <row r="61" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -15543,8 +16206,11 @@
       <c r="BH61">
         <v>3.702</v>
       </c>
+      <c r="BI61" t="s">
+        <v>1443</v>
+      </c>
     </row>
-    <row r="62" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -15719,8 +16385,11 @@
       <c r="BH62">
         <v>3.8029999999999999</v>
       </c>
+      <c r="BI62" t="s">
+        <v>1444</v>
+      </c>
     </row>
-    <row r="63" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -15880,8 +16549,11 @@
       <c r="BH63">
         <v>40.700000000000003</v>
       </c>
+      <c r="BI63" t="s">
+        <v>1445</v>
+      </c>
     </row>
-    <row r="64" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -16059,8 +16731,11 @@
       <c r="BH64">
         <v>3.052</v>
       </c>
+      <c r="BI64" t="s">
+        <v>1446</v>
+      </c>
     </row>
-    <row r="65" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -16223,8 +16898,11 @@
       <c r="BH65">
         <v>4.3559999999999999</v>
       </c>
+      <c r="BI65" t="s">
+        <v>1447</v>
+      </c>
     </row>
-    <row r="66" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -16399,8 +17077,11 @@
       <c r="BH66">
         <v>3.7</v>
       </c>
+      <c r="BI66" t="s">
+        <v>1448</v>
+      </c>
     </row>
-    <row r="67" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -16560,8 +17241,11 @@
       <c r="BH67">
         <v>2</v>
       </c>
+      <c r="BI67" t="s">
+        <v>1449</v>
+      </c>
     </row>
-    <row r="68" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -16739,8 +17423,11 @@
       <c r="BH68">
         <v>4.0999999999999996</v>
       </c>
+      <c r="BI68" t="s">
+        <v>1450</v>
+      </c>
     </row>
-    <row r="69" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -16918,8 +17605,11 @@
       <c r="BH69">
         <v>2.54</v>
       </c>
+      <c r="BI69" t="s">
+        <v>1451</v>
+      </c>
     </row>
-    <row r="70" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -17094,8 +17784,11 @@
       <c r="BH70">
         <v>2.7690000000000001</v>
       </c>
+      <c r="BI70" t="s">
+        <v>1452</v>
+      </c>
     </row>
-    <row r="71" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -17270,8 +17963,11 @@
       <c r="BH71">
         <v>8.1</v>
       </c>
+      <c r="BI71" t="s">
+        <v>1453</v>
+      </c>
     </row>
-    <row r="72" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -17449,8 +18145,11 @@
       <c r="BH72">
         <v>94.2</v>
       </c>
+      <c r="BI72" t="s">
+        <v>1454</v>
+      </c>
     </row>
-    <row r="73" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -17625,8 +18324,11 @@
       <c r="BH73">
         <v>2.2000000000000002</v>
       </c>
+      <c r="BI73" t="s">
+        <v>1455</v>
+      </c>
     </row>
-    <row r="74" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -17801,8 +18503,11 @@
       <c r="BH74">
         <v>23.8</v>
       </c>
+      <c r="BI74" t="s">
+        <v>1456</v>
+      </c>
     </row>
-    <row r="75" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -17974,8 +18679,11 @@
       <c r="BH75">
         <v>1.8</v>
       </c>
+      <c r="BI75" t="s">
+        <v>1457</v>
+      </c>
     </row>
-    <row r="76" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -18135,8 +18843,11 @@
       <c r="BH76">
         <v>0.1</v>
       </c>
+      <c r="BI76" t="s">
+        <v>1458</v>
+      </c>
     </row>
-    <row r="77" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -18314,8 +19025,11 @@
       <c r="BH77">
         <v>2.7</v>
       </c>
+      <c r="BI77" t="s">
+        <v>1459</v>
+      </c>
     </row>
-    <row r="78" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -18490,8 +19204,11 @@
       <c r="BH78">
         <v>40.9</v>
       </c>
+      <c r="BI78" t="s">
+        <v>1460</v>
+      </c>
     </row>
-    <row r="79" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -18654,8 +19371,11 @@
       <c r="BH79">
         <v>2</v>
       </c>
+      <c r="BI79" t="s">
+        <v>1461</v>
+      </c>
     </row>
-    <row r="80" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -18827,8 +19547,11 @@
       <c r="BH80">
         <v>11.7</v>
       </c>
+      <c r="BI80" t="s">
+        <v>1462</v>
+      </c>
     </row>
-    <row r="81" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -19006,8 +19729,11 @@
       <c r="BH81">
         <v>1.8</v>
       </c>
+      <c r="BI81" t="s">
+        <v>1463</v>
+      </c>
     </row>
-    <row r="82" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -19176,8 +19902,11 @@
       <c r="BH82">
         <v>15.085699999999999</v>
       </c>
+      <c r="BI82" t="s">
+        <v>1464</v>
+      </c>
     </row>
-    <row r="83" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -19352,8 +20081,11 @@
       <c r="BH83">
         <v>3</v>
       </c>
+      <c r="BI83" t="s">
+        <v>1465</v>
+      </c>
     </row>
-    <row r="84" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -19516,8 +20248,11 @@
       <c r="BH84">
         <v>3.4060000000000001</v>
       </c>
+      <c r="BI84" t="s">
+        <v>1466</v>
+      </c>
     </row>
-    <row r="85" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -19689,8 +20424,11 @@
       <c r="BH85">
         <v>2.8</v>
       </c>
+      <c r="BI85" t="s">
+        <v>1467</v>
+      </c>
     </row>
-    <row r="86" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -19871,8 +20609,11 @@
       <c r="BH86">
         <v>28.6</v>
       </c>
+      <c r="BI86" t="s">
+        <v>1468</v>
+      </c>
     </row>
-    <row r="87" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -20047,8 +20788,11 @@
       <c r="BH87">
         <v>39.799999999999997</v>
       </c>
+      <c r="BI87" t="s">
+        <v>1469</v>
+      </c>
     </row>
-    <row r="88" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -20223,8 +20967,11 @@
       <c r="BH88">
         <v>3.8</v>
       </c>
+      <c r="BI88" t="s">
+        <v>1470</v>
+      </c>
     </row>
-    <row r="89" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -20396,8 +21143,11 @@
       <c r="BH89">
         <v>4.7</v>
       </c>
+      <c r="BI89" t="s">
+        <v>1471</v>
+      </c>
     </row>
-    <row r="90" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -20572,8 +21322,11 @@
       <c r="BH90">
         <v>2</v>
       </c>
+      <c r="BI90" t="s">
+        <v>1472</v>
+      </c>
     </row>
-    <row r="91" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -20733,8 +21486,11 @@
       <c r="BH91">
         <v>6.2519999999999998</v>
       </c>
+      <c r="BI91" t="s">
+        <v>1473</v>
+      </c>
     </row>
-    <row r="92" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -20909,8 +21665,11 @@
       <c r="BH92">
         <v>2</v>
       </c>
+      <c r="BI92" t="s">
+        <v>1474</v>
+      </c>
     </row>
-    <row r="93" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -21085,8 +21844,11 @@
       <c r="BH93">
         <v>0.5</v>
       </c>
+      <c r="BI93" t="s">
+        <v>1475</v>
+      </c>
     </row>
-    <row r="94" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -21264,8 +22026,11 @@
       <c r="BH94">
         <v>0.5</v>
       </c>
+      <c r="BI94" t="s">
+        <v>1476</v>
+      </c>
     </row>
-    <row r="95" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -21425,8 +22190,11 @@
       <c r="BH95">
         <v>2</v>
       </c>
+      <c r="BI95" t="s">
+        <v>1477</v>
+      </c>
     </row>
-    <row r="96" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -21601,8 +22369,11 @@
       <c r="BH96">
         <v>4.5</v>
       </c>
+      <c r="BI96" t="s">
+        <v>1478</v>
+      </c>
     </row>
-    <row r="97" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -21777,8 +22548,11 @@
       <c r="BH97">
         <v>14.4</v>
       </c>
+      <c r="BI97" t="s">
+        <v>1479</v>
+      </c>
     </row>
-    <row r="98" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -21953,8 +22727,11 @@
       <c r="BH98">
         <v>5.2</v>
       </c>
+      <c r="BI98" t="s">
+        <v>1480</v>
+      </c>
     </row>
-    <row r="99" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -22132,8 +22909,11 @@
       <c r="BH99">
         <v>43.1</v>
       </c>
+      <c r="BI99" t="s">
+        <v>1481</v>
+      </c>
     </row>
-    <row r="100" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -22296,8 +23076,11 @@
       <c r="BH100">
         <v>27.3</v>
       </c>
+      <c r="BI100" t="s">
+        <v>1482</v>
+      </c>
     </row>
-    <row r="101" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -22460,8 +23243,11 @@
       <c r="BH101">
         <v>1.4950000000000001</v>
       </c>
+      <c r="BI101" t="s">
+        <v>1483</v>
+      </c>
     </row>
-    <row r="102" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -22636,8 +23422,11 @@
       <c r="BH102">
         <v>0.8</v>
       </c>
+      <c r="BI102" t="s">
+        <v>1484</v>
+      </c>
     </row>
-    <row r="103" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -22815,8 +23604,11 @@
       <c r="BH103">
         <v>4.4000000000000004</v>
       </c>
+      <c r="BI103" t="s">
+        <v>1439</v>
+      </c>
     </row>
-    <row r="104" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -22979,8 +23771,11 @@
       <c r="BH104">
         <v>4.2</v>
       </c>
+      <c r="BI104" t="s">
+        <v>1485</v>
+      </c>
     </row>
-    <row r="105" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -23146,8 +23941,11 @@
       <c r="BH105">
         <v>3.2949999999999999</v>
       </c>
+      <c r="BI105" t="s">
+        <v>1486</v>
+      </c>
     </row>
-    <row r="106" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -23310,8 +24108,11 @@
       <c r="BH106">
         <v>2</v>
       </c>
+      <c r="BI106" t="s">
+        <v>1487</v>
+      </c>
     </row>
-    <row r="107" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -23474,8 +24275,11 @@
       <c r="BH107">
         <v>16.2</v>
       </c>
+      <c r="BI107" t="s">
+        <v>1488</v>
+      </c>
     </row>
-    <row r="108" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -23641,8 +24445,11 @@
       <c r="BH108">
         <v>6.0659999999999998</v>
       </c>
+      <c r="BI108" t="s">
+        <v>1489</v>
+      </c>
     </row>
-    <row r="109" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -23820,8 +24627,11 @@
       <c r="BH109">
         <v>6.8010000000000002</v>
       </c>
+      <c r="BI109" t="s">
+        <v>1490</v>
+      </c>
     </row>
-    <row r="110" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -23996,8 +24806,11 @@
       <c r="BH110">
         <v>2.7</v>
       </c>
+      <c r="BI110" t="s">
+        <v>1491</v>
+      </c>
     </row>
-    <row r="111" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -24169,8 +24982,11 @@
       <c r="BH111">
         <v>11.8</v>
       </c>
+      <c r="BI111" t="s">
+        <v>1492</v>
+      </c>
     </row>
-    <row r="112" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -24348,8 +25164,11 @@
       <c r="BH112">
         <v>2.4</v>
       </c>
+      <c r="BI112" t="s">
+        <v>1493</v>
+      </c>
     </row>
-    <row r="113" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -24527,8 +25346,11 @@
       <c r="BH113">
         <v>3.24</v>
       </c>
+      <c r="BI113" t="s">
+        <v>1494</v>
+      </c>
     </row>
-    <row r="114" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -24700,8 +25522,11 @@
       <c r="BH114">
         <v>2.1</v>
       </c>
+      <c r="BI114" t="s">
+        <v>1495</v>
+      </c>
     </row>
-    <row r="115" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -24873,8 +25698,11 @@
       <c r="BH115">
         <v>1.64</v>
       </c>
+      <c r="BI115" t="s">
+        <v>1496</v>
+      </c>
     </row>
-    <row r="116" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -25046,8 +25874,11 @@
       <c r="BH116">
         <v>5.4</v>
       </c>
+      <c r="BI116" t="s">
+        <v>1497</v>
+      </c>
     </row>
-    <row r="117" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -25225,8 +26056,11 @@
       <c r="BH117">
         <v>2</v>
       </c>
+      <c r="BI117" t="s">
+        <v>1498</v>
+      </c>
     </row>
-    <row r="118" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -25401,8 +26235,11 @@
       <c r="BH118">
         <v>3.1829999999999998</v>
       </c>
+      <c r="BI118" t="s">
+        <v>1499</v>
+      </c>
     </row>
-    <row r="119" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -25577,8 +26414,11 @@
       <c r="BH119">
         <v>2</v>
       </c>
+      <c r="BI119" t="s">
+        <v>1500</v>
+      </c>
     </row>
-    <row r="120" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -25744,8 +26584,11 @@
       <c r="BH120">
         <v>5.7720000000000002</v>
       </c>
+      <c r="BI120" t="s">
+        <v>1501</v>
+      </c>
     </row>
-    <row r="121" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -25908,8 +26751,11 @@
       <c r="BH121">
         <v>3.6669999999999998</v>
       </c>
+      <c r="BI121" t="s">
+        <v>1502</v>
+      </c>
     </row>
-    <row r="122" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -26066,8 +26912,11 @@
       <c r="BH122">
         <v>1.6</v>
       </c>
+      <c r="BI122" t="s">
+        <v>1439</v>
+      </c>
     </row>
-    <row r="123" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -26227,8 +27076,11 @@
       <c r="BH123">
         <v>1.3</v>
       </c>
+      <c r="BI123" t="s">
+        <v>1503</v>
+      </c>
     </row>
-    <row r="124" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -26403,8 +27255,11 @@
       <c r="BH124">
         <v>0.9</v>
       </c>
+      <c r="BI124" t="s">
+        <v>1504</v>
+      </c>
     </row>
-    <row r="125" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -26582,8 +27437,11 @@
       <c r="BH125">
         <v>1.89</v>
       </c>
+      <c r="BI125" t="s">
+        <v>1505</v>
+      </c>
     </row>
-    <row r="126" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -26746,8 +27604,11 @@
       <c r="BH126">
         <v>2.3809999999999998</v>
       </c>
+      <c r="BI126" t="s">
+        <v>1506</v>
+      </c>
     </row>
-    <row r="127" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -26925,8 +27786,11 @@
       <c r="BH127">
         <v>2.0369999999999999</v>
       </c>
+      <c r="BI127" t="s">
+        <v>1507</v>
+      </c>
     </row>
-    <row r="128" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -27101,8 +27965,11 @@
       <c r="BH128">
         <v>2.7970000000000002</v>
       </c>
+      <c r="BI128" t="s">
+        <v>1508</v>
+      </c>
     </row>
-    <row r="129" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -27265,8 +28132,11 @@
       <c r="BH129">
         <v>0.2</v>
       </c>
+      <c r="BI129" t="s">
+        <v>1509</v>
+      </c>
     </row>
-    <row r="130" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -27441,8 +28311,11 @@
       <c r="BH130">
         <v>1.8</v>
       </c>
+      <c r="BI130" t="s">
+        <v>1510</v>
+      </c>
     </row>
-    <row r="131" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -27599,8 +28472,11 @@
       <c r="BH131">
         <v>4.258</v>
       </c>
+      <c r="BI131" t="s">
+        <v>1511</v>
+      </c>
     </row>
-    <row r="132" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -27775,8 +28651,11 @@
       <c r="BH132">
         <v>0.9</v>
       </c>
+      <c r="BI132" t="s">
+        <v>1512</v>
+      </c>
     </row>
-    <row r="133" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -27936,8 +28815,11 @@
       <c r="BH133">
         <v>2.4870000000000001</v>
       </c>
+      <c r="BI133" t="s">
+        <v>1513</v>
+      </c>
     </row>
-    <row r="134" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -28112,8 +28994,11 @@
       <c r="BH134">
         <v>3.9049999999999998</v>
       </c>
+      <c r="BI134" t="s">
+        <v>1514</v>
+      </c>
     </row>
-    <row r="135" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -28276,8 +29161,11 @@
       <c r="BH135">
         <v>3.2959999999999998</v>
       </c>
+      <c r="BI135" t="s">
+        <v>1515</v>
+      </c>
     </row>
-    <row r="136" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -28455,8 +29343,11 @@
       <c r="BH136">
         <v>2.8</v>
       </c>
+      <c r="BI136" t="s">
+        <v>1516</v>
+      </c>
     </row>
-    <row r="137" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -28631,8 +29522,11 @@
       <c r="BH137">
         <v>2.3740000000000001</v>
       </c>
+      <c r="BI137" t="s">
+        <v>1517</v>
+      </c>
     </row>
-    <row r="138" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -28795,8 +29689,11 @@
       <c r="BH138">
         <v>1.8</v>
       </c>
+      <c r="BI138" t="s">
+        <v>1518</v>
+      </c>
     </row>
-    <row r="139" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -28974,8 +29871,11 @@
       <c r="BH139">
         <v>0.1</v>
       </c>
+      <c r="BI139" t="s">
+        <v>1519</v>
+      </c>
     </row>
-    <row r="140" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -29141,8 +30041,11 @@
       <c r="BH140">
         <v>0.9</v>
       </c>
+      <c r="BI140" t="s">
+        <v>1439</v>
+      </c>
     </row>
-    <row r="141" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -29320,8 +30223,11 @@
       <c r="BH141">
         <v>5.1379999999999999</v>
       </c>
+      <c r="BI141" t="s">
+        <v>1520</v>
+      </c>
     </row>
-    <row r="142" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -29496,8 +30402,11 @@
       <c r="BH142">
         <v>6.7</v>
       </c>
+      <c r="BI142" t="s">
+        <v>1521</v>
+      </c>
     </row>
-    <row r="143" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -29660,8 +30569,11 @@
       <c r="BH143">
         <v>0.1</v>
       </c>
+      <c r="BI143" t="s">
+        <v>1522</v>
+      </c>
     </row>
-    <row r="144" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -29827,8 +30739,11 @@
       <c r="BH144">
         <v>0.1</v>
       </c>
+      <c r="BI144" t="s">
+        <v>1523</v>
+      </c>
     </row>
-    <row r="145" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -30003,8 +30918,11 @@
       <c r="BH145">
         <v>4.4000000000000004</v>
       </c>
+      <c r="BI145" t="s">
+        <v>1524</v>
+      </c>
     </row>
-    <row r="146" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -30173,8 +31091,11 @@
       <c r="BH146">
         <v>2.5</v>
       </c>
+      <c r="BI146" t="s">
+        <v>1439</v>
+      </c>
     </row>
-    <row r="147" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -30337,8 +31258,11 @@
       <c r="BH147">
         <v>4.7590000000000003</v>
       </c>
+      <c r="BI147" t="s">
+        <v>1525</v>
+      </c>
     </row>
-    <row r="148" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -30513,8 +31437,11 @@
       <c r="BH148">
         <v>2.532</v>
       </c>
+      <c r="BI148" t="s">
+        <v>1526</v>
+      </c>
     </row>
-    <row r="149" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -30689,8 +31616,11 @@
       <c r="BH149">
         <v>3.67</v>
       </c>
+      <c r="BI149" t="s">
+        <v>1527</v>
+      </c>
     </row>
-    <row r="150" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -30868,8 +31798,11 @@
       <c r="BH150">
         <v>5.4859999999999998</v>
       </c>
+      <c r="BI150" t="s">
+        <v>1528</v>
+      </c>
     </row>
-    <row r="151" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -31047,8 +31980,11 @@
       <c r="BH151">
         <v>2</v>
       </c>
+      <c r="BI151" t="s">
+        <v>1529</v>
+      </c>
     </row>
-    <row r="152" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -31208,8 +32144,11 @@
       <c r="BH152">
         <v>1.96</v>
       </c>
+      <c r="BI152" t="s">
+        <v>1530</v>
+      </c>
     </row>
-    <row r="153" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -31387,8 +32326,11 @@
       <c r="BH153">
         <v>3.23</v>
       </c>
+      <c r="BI153" t="s">
+        <v>1531</v>
+      </c>
     </row>
-    <row r="154" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -31563,8 +32505,11 @@
       <c r="BH154">
         <v>13.8</v>
       </c>
+      <c r="BI154" t="s">
+        <v>1532</v>
+      </c>
     </row>
-    <row r="155" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -31730,8 +32675,11 @@
       <c r="BH155">
         <v>3.4620000000000002</v>
       </c>
+      <c r="BI155" t="s">
+        <v>1533</v>
+      </c>
     </row>
-    <row r="156" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -31894,8 +32842,11 @@
       <c r="BH156">
         <v>7.0810000000000004</v>
       </c>
+      <c r="BI156" t="s">
+        <v>1534</v>
+      </c>
     </row>
-    <row r="157" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -32073,8 +33024,11 @@
       <c r="BH157">
         <v>9.6</v>
       </c>
+      <c r="BI157" t="s">
+        <v>1535</v>
+      </c>
     </row>
-    <row r="158" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -32252,8 +33206,11 @@
       <c r="BH158">
         <v>3.13</v>
       </c>
+      <c r="BI158" t="s">
+        <v>1536</v>
+      </c>
     </row>
-    <row r="159" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -32419,8 +33376,11 @@
       <c r="BH159">
         <v>4.4000000000000004</v>
       </c>
+      <c r="BI159" t="s">
+        <v>1537</v>
+      </c>
     </row>
-    <row r="160" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -32586,8 +33546,11 @@
       <c r="BH160">
         <v>16.3</v>
       </c>
+      <c r="BI160" t="s">
+        <v>1538</v>
+      </c>
     </row>
-    <row r="161" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -32765,8 +33728,11 @@
       <c r="BH161">
         <v>12</v>
       </c>
+      <c r="BI161" t="s">
+        <v>1539</v>
+      </c>
     </row>
-    <row r="162" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -32941,8 +33907,11 @@
       <c r="BH162">
         <v>1.923</v>
       </c>
+      <c r="BI162" t="s">
+        <v>1540</v>
+      </c>
     </row>
-    <row r="163" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -33105,8 +34074,11 @@
       <c r="BH163">
         <v>3.121</v>
       </c>
+      <c r="BI163" t="s">
+        <v>1541</v>
+      </c>
     </row>
-    <row r="164" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -33284,8 +34256,11 @@
       <c r="BH164">
         <v>8.9</v>
       </c>
+      <c r="BI164" t="s">
+        <v>1542</v>
+      </c>
     </row>
-    <row r="165" spans="1:60" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -33459,6 +34434,9 @@
       </c>
       <c r="BH165">
         <v>3.4</v>
+      </c>
+      <c r="BI165" t="s">
+        <v>1543</v>
       </c>
     </row>
   </sheetData>

</xml_diff>